<commit_message>
chore: updated the mistaken document
</commit_message>
<xml_diff>
--- a/Developer/Bibek KC/Individual Timesheet Bibek KC_S394325.xlsx
+++ b/Developer/Bibek KC/Individual Timesheet Bibek KC_S394325.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NestedDisk\Semester_3\Software_Engineering_Practise\SoftwareEngineeringPractise\Bibek KC\Individual_Timesheet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\NestedDisk\Semester_3\Software_Engineering_Practise\SoftwareEngineeringPractise\Developer\Bibek KC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BD0A53-C465-4C7B-B653-6D4C105C6E3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35B12B21-C6A0-40E7-8936-EF61A4EA952A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="38">
   <si>
     <t>Week</t>
   </si>
@@ -141,6 +141,18 @@
   </si>
   <si>
     <t>Debugging and testing of the code using selenium</t>
+  </si>
+  <si>
+    <t>Week 8</t>
+  </si>
+  <si>
+    <t>Meeting and debugging of the code</t>
+  </si>
+  <si>
+    <t>Postman API testing of the code</t>
+  </si>
+  <si>
+    <t>Research on quality code and folder structure</t>
   </si>
 </sst>
 </file>
@@ -513,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="12.54296875" customWidth="1"/>
@@ -936,6 +948,62 @@
         <v>33</v>
       </c>
     </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
+      <c r="E30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31">
+        <v>2</v>
+      </c>
+      <c r="E31" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32" t="s">
+        <v>16</v>
+      </c>
+      <c r="D32">
+        <v>2</v>
+      </c>
+      <c r="E32" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>